<commit_message>
updated filter file for power-only NA runs
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_NorthAmerica.xlsx
+++ b/Conversion Script/Set_filter_file_NorthAmerica.xlsx
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -2430,7 +2430,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2450,7 +2450,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -2470,7 +2470,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2480,7 +2480,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -2490,7 +2490,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -2500,7 +2500,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2510,7 +2510,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2520,7 +2520,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2540,7 +2540,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2550,7 +2550,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -2560,7 +2560,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -2630,7 +2630,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -2650,7 +2650,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -2660,7 +2660,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -2680,7 +2680,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -2690,7 +2690,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2720,7 +2720,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2740,7 +2740,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -2750,7 +2750,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -2770,7 +2770,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2780,7 +2780,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2830,7 +2830,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2840,7 +2840,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2860,7 +2860,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2870,7 +2870,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2890,7 +2890,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -2900,7 +2900,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -3240,7 +3240,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -3250,7 +3250,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -3260,7 +3260,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115">
@@ -3270,7 +3270,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -3280,7 +3280,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -3310,7 +3310,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -3320,7 +3320,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
@@ -3330,7 +3330,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -3340,7 +3340,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="123">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -3370,7 +3370,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -3380,7 +3380,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">
@@ -3390,7 +3390,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
@@ -3400,7 +3400,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -3410,7 +3410,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -3420,7 +3420,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -3440,7 +3440,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -3450,7 +3450,7 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -3460,7 +3460,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135">
@@ -3470,7 +3470,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -3480,7 +3480,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -3490,7 +3490,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -3500,7 +3500,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -3510,7 +3510,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -3550,7 +3550,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -3560,7 +3560,7 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146">
@@ -3580,7 +3580,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -3590,7 +3590,7 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -3620,7 +3620,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -3650,7 +3650,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154">
@@ -3660,7 +3660,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3739,7 +3739,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3759,7 +3759,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3769,7 +3769,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3779,7 +3779,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3833,7 +3833,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -3903,7 +3903,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -3943,7 +3943,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3953,7 +3953,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3963,7 +3963,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3973,7 +3973,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -3983,7 +3983,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -4003,7 +4003,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -4033,7 +4033,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4043,7 +4043,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -4053,7 +4053,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4073,7 +4073,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -4103,7 +4103,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -4113,7 +4113,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4143,7 +4143,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -4153,7 +4153,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added steam turbines to NA data set filter file
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_NorthAmerica.xlsx
+++ b/Conversion Script/Set_filter_file_NorthAmerica.xlsx
@@ -2386,7 +2386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B159"/>
+  <dimension ref="A1:B160"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3317,7 +3317,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>P_Geothermal</t>
+          <t>P_Gas_Steam</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -3327,7 +3327,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>P_H2_OCGT</t>
+          <t>P_Geothermal</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -3337,7 +3337,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>P_Hydro_Reservoir</t>
+          <t>P_H2_OCGT</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -3347,7 +3347,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>P_Hydro_RoR</t>
+          <t>P_Hydro_Reservoir</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -3357,7 +3357,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>P_Nuclear</t>
+          <t>P_Hydro_RoR</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -3367,7 +3367,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>P_Ocean</t>
+          <t>P_Nuclear</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -3377,7 +3377,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>P_Oil</t>
+          <t>P_Ocean</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -3387,7 +3387,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>P_PV_Rooftop_Commercial</t>
+          <t>P_Oil</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -3397,7 +3397,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>P_PV_Rooftop_Residential</t>
+          <t>P_PV_Rooftop_Commercial</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -3407,7 +3407,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>P_PV_Utility_Avg</t>
+          <t>P_PV_Rooftop_Residential</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -3417,7 +3417,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>P_PV_Utility_Inf</t>
+          <t>P_PV_Utility_Avg</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -3427,7 +3427,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>P_PV_Utility_Opt</t>
+          <t>P_PV_Utility_Inf</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -3437,7 +3437,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>P_PV_Utility_Tracking</t>
+          <t>P_PV_Utility_Opt</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -3447,7 +3447,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>P_Wind_Offshore_Deep</t>
+          <t>P_PV_Utility_Tracking</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -3457,7 +3457,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>P_Wind_Offshore_Shallow</t>
+          <t>P_Wind_Offshore_Deep</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -3467,7 +3467,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>P_Wind_Offshore_Transitional</t>
+          <t>P_Wind_Offshore_Shallow</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -3477,7 +3477,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>P_Wind_Onshore_Avg</t>
+          <t>P_Wind_Offshore_Transitional</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -3487,7 +3487,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>P_Wind_Onshore_Inf</t>
+          <t>P_Wind_Onshore_Avg</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -3497,27 +3497,27 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
+          <t>P_Wind_Onshore_Inf</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
           <t>P_Wind_Onshore_Opt</t>
         </is>
       </c>
-      <c r="B111" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>PSNG_Air_Bio</t>
-        </is>
-      </c>
       <c r="B112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Air_Conv</t>
+          <t>PSNG_Air_Bio</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -3527,7 +3527,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Air_H2</t>
+          <t>PSNG_Air_Conv</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -3537,7 +3537,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Rail_Conv</t>
+          <t>PSNG_Air_H2</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -3547,7 +3547,7 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Rail_Electric</t>
+          <t>PSNG_Rail_Conv</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -3557,7 +3557,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Road_BEV</t>
+          <t>PSNG_Rail_Electric</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -3567,7 +3567,7 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Road_H2</t>
+          <t>PSNG_Road_BEV</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -3577,7 +3577,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Road_ICE</t>
+          <t>PSNG_Road_H2</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -3587,7 +3587,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>PSNG_Road_LNG</t>
+          <t>PSNG_Road_ICE</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -3597,17 +3597,17 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
+          <t>PSNG_Road_LNG</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
           <t>PSNG_Road_PHEV</t>
-        </is>
-      </c>
-      <c r="B121" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>R_Biogas</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -3617,7 +3617,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>R_Coal_Hardcoal</t>
+          <t>R_Biogas</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -3627,7 +3627,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>R_Coal_Lignite</t>
+          <t>R_Coal_Hardcoal</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -3637,7 +3637,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>R_Gas</t>
+          <t>R_Coal_Lignite</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -3647,7 +3647,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>R_Grass</t>
+          <t>R_Gas</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -3657,7 +3657,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>R_Nuclear</t>
+          <t>R_Grass</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -3667,7 +3667,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>R_Oil</t>
+          <t>R_Nuclear</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -3677,7 +3677,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>R_Paper_Cardboard</t>
+          <t>R_Oil</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -3687,7 +3687,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>R_Residues</t>
+          <t>R_Paper_Cardboard</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -3697,7 +3697,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>R_Roundwood</t>
+          <t>R_Residues</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -3707,7 +3707,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>R_Waste</t>
+          <t>R_Roundwood</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -3717,7 +3717,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>R_Wood</t>
+          <t>R_Waste</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -3727,7 +3727,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>X_Alkaline_Electrolysis</t>
+          <t>R_Wood</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -3737,7 +3737,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>X_ATR_CCS</t>
+          <t>X_Alkaline_Electrolysis</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -3747,7 +3747,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>X_Biofuel</t>
+          <t>X_ATR_CCS</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -3757,17 +3757,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>X_Biofuel</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
           <t>X_Convert_HD</t>
-        </is>
-      </c>
-      <c r="B137" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>X_DAC_HT</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -3777,27 +3777,27 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
+          <t>X_DAC_HT</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
           <t>X_DAC_LT</t>
         </is>
       </c>
-      <c r="B139" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
+      <c r="B140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
         <is>
           <t>X_Electrolysis</t>
-        </is>
-      </c>
-      <c r="B140" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>X_Gasifier</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -3807,17 +3807,17 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
+          <t>X_Gasifier</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
           <t>X_Liquifier</t>
-        </is>
-      </c>
-      <c r="B142" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>X_Methanation</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -3827,7 +3827,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>X_PEM_Electrolysis</t>
+          <t>X_Methanation</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -3837,7 +3837,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>X_Powerfuel</t>
+          <t>X_PEM_Electrolysis</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -3847,7 +3847,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>X_SMR</t>
+          <t>X_Powerfuel</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -3857,7 +3857,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>X_SOEC_Electrolysis</t>
+          <t>X_SMR</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -3867,7 +3867,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Z_ETS_Buy</t>
+          <t>X_SOEC_Electrolysis</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -3877,7 +3877,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Z_ETS_Sell</t>
+          <t>Z_ETS_Buy</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -3887,27 +3887,27 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
+          <t>Z_ETS_Sell</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
           <t>Z_Import_Gas</t>
         </is>
       </c>
-      <c r="B150" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+      <c r="B151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>Z_Import_H2</t>
-        </is>
-      </c>
-      <c r="B151" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Z_Import_Hardcoal</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -3917,7 +3917,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Z_Import_LNG</t>
+          <t>Z_Import_Hardcoal</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -3927,7 +3927,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Z_Import_Oil</t>
+          <t>Z_Import_LNG</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -3937,17 +3937,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>X_Convert_Power</t>
+          <t>Z_Import_Oil</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>P_EGS_R1</t>
+          <t>X_Convert_Power</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -3957,7 +3957,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>P_EGS_R2</t>
+          <t>P_EGS_R1</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -3967,7 +3967,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>P_EGS_R3</t>
+          <t>P_EGS_R2</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -3977,10 +3977,20 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
+          <t>P_EGS_R3</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
           <t>P_EGS_R4</t>
         </is>
       </c>
-      <c r="B159" t="n">
+      <c r="B160" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(na): register P_Gas_CCGT_Residual in NA conversion filters + doc
- Add P_Gas_CCGT_Residual = 1 to the Technology_selection sheet of
  Set_filter_file_NorthAmerica.xlsx and Set_filter_file_NorthAmerica_allFuels.xlsx
  (a tech absent from the filter is dropped by master_function, so the model would
  never see the new CCGT residual tech).
- CLAUDE.md: document that new set members (technology, region, fuel, ...) must
  also be added to the matching *_selection sheet of every Set_filter_file*.xlsx.

Note: the .xlsx are binary, so this also carries prior uncommitted NA filter edits
that could not be isolated from the P_Gas_CCGT_Residual addition.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_NorthAmerica.xlsx
+++ b/Conversion Script/Set_filter_file_NorthAmerica.xlsx
@@ -2386,7 +2386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B160"/>
+  <dimension ref="A1:B162"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3991,6 +3991,26 @@
         </is>
       </c>
       <c r="B160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>P_Nuclear_SMR</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>P_Gas_CCGT_Residual</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>